<commit_message>
Daily iteration 2026-07-18: fixed truncated literature_gap_data.json + atomic-write hardening in gap_analysis_daily.py; re-validated dapagliflozin nephropathy+T2D (PMID 38730538 NDT-2024); credibility sweep clean; pipeline 41/41 OK
</commit_message>
<xml_diff>
--- a/Diabetes_Research_Tracker.xlsx
+++ b/Diabetes_Research_Tracker.xlsx
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Orforglipron</t>
+          <t>Orforglipron (Foundayo)</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
@@ -1758,27 +1758,27 @@
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>Oral GLP-1 receptor agonist</t>
+          <t>Oral non-peptide GLP-1 receptor agonist</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>FDA Approved (Apr 1, 2026)</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>Oral glucose + weight</t>
+          <t>Glycemic control / weight management</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
-          <t>Oral GLP-1; superior to oral semaglutide in ACHIEVE-3 (Lancet Feb 2026); NDA submitted; FDA target action date Apr 10, 2026</t>
+          <t>First oral small-molecule GLP-1 RA. Superior to oral semaglutide in ACHIEVE-3 (Lancet Feb 2026). FDA approved Apr 1, 2026 under CNPV ~294 days ahead of PDUFA; no food/water/timing restrictions. T2D indication in development.</t>
         </is>
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>NDA Under Review</t>
+          <t>FDA Approved</t>
         </is>
       </c>
       <c r="J22" s="15" t="n">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="K22" s="16" t="inlineStr">
         <is>
-          <t>https://www.diabetesincontrol.com/top-7-breakthroughs-in-type-2-diabetes-treatment-for-2025/</t>
+          <t>https://investor.lilly.com/news-releases/news-release-details/fda-approves-lillys-foundayotm-orforglipron-only-glp-1-pill</t>
         </is>
       </c>
     </row>
@@ -4328,37 +4328,37 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>Oral GLP-1</t>
+          <t>Biosimilar</t>
         </is>
       </c>
       <c r="C69" s="25" t="inlineStr">
         <is>
-          <t>Foundayo (Orforglipron)</t>
+          <t>Merilog (Biosimilar Insulin Aspart)</t>
         </is>
       </c>
       <c r="D69" s="25" t="inlineStr">
         <is>
-          <t>Eli Lilly</t>
+          <t>FDA-approved biosimilar</t>
         </is>
       </c>
       <c r="E69" s="25" t="inlineStr">
         <is>
-          <t>Oral non-peptide GLP-1 receptor agonist</t>
+          <t>Biosimilar of insulin aspart (Novolog)</t>
         </is>
       </c>
       <c r="F69" s="25" t="inlineStr">
         <is>
-          <t>FDA Approved (Apr 1, 2026)</t>
+          <t>FDA Approved (Mar 2026)</t>
         </is>
       </c>
       <c r="G69" s="25" t="inlineStr">
         <is>
-          <t>Obesity/overweight (T2D indication pending)</t>
+          <t>Diabetes (T1D/T2D)</t>
         </is>
       </c>
       <c r="H69" s="25" t="inlineStr">
         <is>
-          <t>First oral non-peptide GLP-1 pill; approved under CNPV program 294 days ahead of PDUFA; any time of day dosing without food/water restrictions</t>
+          <t>Biosimilar insulin aspart; expands insulin access options</t>
         </is>
       </c>
       <c r="I69" s="25" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="K69" s="25" t="inlineStr">
         <is>
-          <t>https://www.hcplive.com/view/diabetes-dialogue-orforglipron-receives-fda-approval-for-chronic-weight-management</t>
+          <t>https://www.hcplive.com/view/fda-approves-merilog-biosimilar-product-insulin-aspart-novolog-diabetes</t>
         </is>
       </c>
     </row>
@@ -4383,37 +4383,37 @@
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>Biosimilar</t>
+          <t>Novel Insulin</t>
         </is>
       </c>
       <c r="C70" s="25" t="inlineStr">
         <is>
-          <t>Merilog (Biosimilar Insulin Aspart)</t>
+          <t>Awiqli (Insulin Icodec)</t>
         </is>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>FDA-approved biosimilar</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E70" s="25" t="inlineStr">
         <is>
-          <t>Biosimilar of insulin aspart (Novolog)</t>
+          <t>Once-weekly basal insulin</t>
         </is>
       </c>
       <c r="F70" s="25" t="inlineStr">
         <is>
-          <t>FDA Approved (Mar 2026)</t>
+          <t>FDA Approved (Mar 27, 2026)</t>
         </is>
       </c>
       <c r="G70" s="25" t="inlineStr">
         <is>
-          <t>Diabetes (T1D/T2D)</t>
+          <t>T2D glycemic control</t>
         </is>
       </c>
       <c r="H70" s="25" t="inlineStr">
         <is>
-          <t>Biosimilar insulin aspart; expands insulin access options</t>
+          <t>First once-weekly basal insulin; reduces injections from 7 to 1 per week; nationwide availability H2 2026</t>
         </is>
       </c>
       <c r="I70" s="25" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="K70" s="25" t="inlineStr">
         <is>
-          <t>https://www.hcplive.com/view/fda-approves-merilog-biosimilar-product-insulin-aspart-novolog-diabetes</t>
+          <t>https://www.roi-nj.com/2026/04/02/healthcare/fda-approves-novo-nordisks-awiqli-a-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes/</t>
         </is>
       </c>
     </row>
@@ -4438,37 +4438,37 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>Novel Insulin</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="C71" s="25" t="inlineStr">
         <is>
-          <t>Awiqli (Insulin Icodec)</t>
+          <t>MiniMed Flex AID System</t>
         </is>
       </c>
       <c r="D71" s="25" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Medtronic</t>
         </is>
       </c>
       <c r="E71" s="25" t="inlineStr">
         <is>
-          <t>Once-weekly basal insulin</t>
+          <t>Automated insulin delivery system</t>
         </is>
       </c>
       <c r="F71" s="25" t="inlineStr">
         <is>
-          <t>FDA Approved (Mar 27, 2026)</t>
+          <t>FDA Cleared (Mar 18, 2026)</t>
         </is>
       </c>
       <c r="G71" s="25" t="inlineStr">
         <is>
-          <t>T2D glycemic control</t>
+          <t>T1D (≥7yr) and insulin-requiring T2D</t>
         </is>
       </c>
       <c r="H71" s="25" t="inlineStr">
         <is>
-          <t>First once-weekly basal insulin; reduces injections from 7 to 1 per week; nationwide availability H2 2026</t>
+          <t>New AID system cleared for ages ≥7 with T1D and adults with insulin-requiring T2D</t>
         </is>
       </c>
       <c r="I71" s="25" t="inlineStr">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="K71" s="25" t="inlineStr">
         <is>
-          <t>https://www.roi-nj.com/2026/04/02/healthcare/fda-approves-novo-nordisks-awiqli-a-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes/</t>
+          <t>https://news.medtronic.com/</t>
         </is>
       </c>
     </row>
@@ -4493,42 +4493,42 @@
       </c>
       <c r="B72" s="25" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Novel Mechanism</t>
         </is>
       </c>
       <c r="C72" s="25" t="inlineStr">
         <is>
-          <t>MiniMed Flex AID System</t>
+          <t>Icovamenib (Biomea Fusion)</t>
         </is>
       </c>
       <c r="D72" s="25" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>Biomea Fusion</t>
         </is>
       </c>
       <c r="E72" s="25" t="inlineStr">
         <is>
-          <t>Automated insulin delivery system</t>
+          <t>Menin inhibitor for beta cell regeneration</t>
         </is>
       </c>
       <c r="F72" s="25" t="inlineStr">
         <is>
-          <t>FDA Cleared (Mar 18, 2026)</t>
+          <t>Phase 2 (NCT07502495, NCT07502508)</t>
         </is>
       </c>
       <c r="G72" s="25" t="inlineStr">
         <is>
-          <t>T1D (≥7yr) and insulin-requiring T2D</t>
+          <t>T2D beta cell restoration</t>
         </is>
       </c>
       <c r="H72" s="25" t="inlineStr">
         <is>
-          <t>New AID system cleared for ages ≥7 with T1D and adults with insulin-requiring T2D</t>
+          <t>Novel menin inhibitor; Phase 2 expansion initiated April 2026</t>
         </is>
       </c>
       <c r="I72" s="25" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Recruiting</t>
         </is>
       </c>
       <c r="J72" s="25" t="n">
@@ -4536,62 +4536,62 @@
       </c>
       <c r="K72" s="25" t="inlineStr">
         <is>
-          <t>https://news.medtronic.com/</t>
+          <t>https://clinicaltrials.gov/study/NCT07502495</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="25" t="inlineStr">
+      <c r="A73" s="26" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B73" s="25" t="inlineStr">
-        <is>
-          <t>Novel Mechanism</t>
-        </is>
-      </c>
-      <c r="C73" s="25" t="inlineStr">
-        <is>
-          <t>Icovamenib (Biomea Fusion)</t>
-        </is>
-      </c>
-      <c r="D73" s="25" t="inlineStr">
-        <is>
-          <t>Biomea Fusion</t>
-        </is>
-      </c>
-      <c r="E73" s="25" t="inlineStr">
-        <is>
-          <t>Menin inhibitor for beta cell regeneration</t>
-        </is>
-      </c>
-      <c r="F73" s="25" t="inlineStr">
-        <is>
-          <t>Phase 2 (NCT07502495, NCT07502508)</t>
-        </is>
-      </c>
-      <c r="G73" s="25" t="inlineStr">
-        <is>
-          <t>T2D beta cell restoration</t>
-        </is>
-      </c>
-      <c r="H73" s="25" t="inlineStr">
-        <is>
-          <t>Novel menin inhibitor; Phase 2 expansion initiated April 2026</t>
-        </is>
-      </c>
-      <c r="I73" s="25" t="inlineStr">
-        <is>
-          <t>Recruiting</t>
-        </is>
-      </c>
-      <c r="J73" s="25" t="n">
+      <c r="B73" s="26" t="inlineStr">
+        <is>
+          <t>Insulin - Weekly Basal</t>
+        </is>
+      </c>
+      <c r="C73" s="26" t="inlineStr">
+        <is>
+          <t>Awiqli (insulin icodec)</t>
+        </is>
+      </c>
+      <c r="D73" s="26" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="E73" s="26" t="inlineStr">
+        <is>
+          <t>Once-weekly basal insulin</t>
+        </is>
+      </c>
+      <c r="F73" s="26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G73" s="26" t="inlineStr">
+        <is>
+          <t>Reduce injection burden</t>
+        </is>
+      </c>
+      <c r="H73" s="26" t="inlineStr">
+        <is>
+          <t>FDA approved March 2026 — first once-weekly basal insulin for T2D. Phase 3 trial NCT07076199 testing in T1D.</t>
+        </is>
+      </c>
+      <c r="I73" s="26" t="inlineStr">
+        <is>
+          <t>FDA Approved (T2D)</t>
+        </is>
+      </c>
+      <c r="J73" s="26" t="n">
         <v>2026</v>
       </c>
-      <c r="K73" s="25" t="inlineStr">
-        <is>
-          <t>https://clinicaltrials.gov/study/NCT07502495</t>
+      <c r="K73" s="26" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/fda-approves-novo-nordisks-awiqli-the-first-and-only-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes-302726839.html</t>
         </is>
       </c>
     </row>
@@ -4603,22 +4603,22 @@
       </c>
       <c r="B74" s="26" t="inlineStr">
         <is>
-          <t>Insulin - Weekly Basal</t>
+          <t>SGLT2i - Generic Access</t>
         </is>
       </c>
       <c r="C74" s="26" t="inlineStr">
         <is>
-          <t>Awiqli (insulin icodec)</t>
+          <t>Generic Dapagliflozin (Farxiga)</t>
         </is>
       </c>
       <c r="D74" s="26" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Multiple (FDA generic approval)</t>
         </is>
       </c>
       <c r="E74" s="26" t="inlineStr">
         <is>
-          <t>Once-weekly basal insulin</t>
+          <t>SGLT2 inhibition</t>
         </is>
       </c>
       <c r="F74" s="26" t="inlineStr">
@@ -4628,17 +4628,17 @@
       </c>
       <c r="G74" s="26" t="inlineStr">
         <is>
-          <t>Reduce injection burden</t>
+          <t>Broaden SGLT2i access</t>
         </is>
       </c>
       <c r="H74" s="26" t="inlineStr">
         <is>
-          <t>FDA approved March 2026 — first once-weekly basal insulin for T2D. Phase 3 trial NCT07076199 testing in T1D.</t>
+          <t>First generics of Farxiga approved April 2026 for HF risk reduction in T2D + glycemic control. Increases access.</t>
         </is>
       </c>
       <c r="I74" s="26" t="inlineStr">
         <is>
-          <t>FDA Approved (T2D)</t>
+          <t>FDA Approved (Generic)</t>
         </is>
       </c>
       <c r="J74" s="26" t="n">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="K74" s="26" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/fda-approves-novo-nordisks-awiqli-the-first-and-only-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes-302726839.html</t>
+          <t>https://www.fda.gov/drugs/drug-alerts-and-statements/fda-approves-first-generic-dapagliflozin-tablets</t>
         </is>
       </c>
     </row>
@@ -4658,22 +4658,22 @@
       </c>
       <c r="B75" s="26" t="inlineStr">
         <is>
-          <t>SGLT2i - Generic Access</t>
+          <t>SGLT2i + Metformin - Generic</t>
         </is>
       </c>
       <c r="C75" s="26" t="inlineStr">
         <is>
-          <t>Generic Dapagliflozin (Farxiga)</t>
+          <t>Generic Dapagliflozin-Metformin</t>
         </is>
       </c>
       <c r="D75" s="26" t="inlineStr">
         <is>
-          <t>Multiple (FDA generic approval)</t>
+          <t>Lupin</t>
         </is>
       </c>
       <c r="E75" s="26" t="inlineStr">
         <is>
-          <t>SGLT2 inhibition</t>
+          <t>SGLT2i + biguanide combo</t>
         </is>
       </c>
       <c r="F75" s="26" t="inlineStr">
@@ -4683,12 +4683,12 @@
       </c>
       <c r="G75" s="26" t="inlineStr">
         <is>
-          <t>Broaden SGLT2i access</t>
+          <t>Lower-cost T2D combo</t>
         </is>
       </c>
       <c r="H75" s="26" t="inlineStr">
         <is>
-          <t>First generics of Farxiga approved April 2026 for HF risk reduction in T2D + glycemic control. Increases access.</t>
+          <t>Lupin FDA approval April 8, 2026. Lower-cost combination for T2D management.</t>
         </is>
       </c>
       <c r="I75" s="26" t="inlineStr">
@@ -4701,34 +4701,34 @@
       </c>
       <c r="K75" s="26" t="inlineStr">
         <is>
-          <t>https://www.fda.gov/drugs/drug-alerts-and-statements/fda-approves-first-generic-dapagliflozin-tablets</t>
+          <t>https://www.prismnews.com/news/lupin-wins-fda-approval-for-generic-dapagliflozin-metformin</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>T2D</t>
+          <t>Cross</t>
         </is>
       </c>
       <c r="B76" s="26" t="inlineStr">
         <is>
-          <t>SGLT2i + Metformin - Generic</t>
+          <t>GLP-1 - Oral</t>
         </is>
       </c>
       <c r="C76" s="26" t="inlineStr">
         <is>
-          <t>Generic Dapagliflozin-Metformin</t>
+          <t>Oral Semaglutide 25mg (Wegovy)</t>
         </is>
       </c>
       <c r="D76" s="26" t="inlineStr">
         <is>
-          <t>Lupin</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E76" s="26" t="inlineStr">
         <is>
-          <t>SGLT2i + biguanide combo</t>
+          <t>Oral GLP-1 RA for weight loss</t>
         </is>
       </c>
       <c r="F76" s="26" t="inlineStr">
@@ -4738,17 +4738,17 @@
       </c>
       <c r="G76" s="26" t="inlineStr">
         <is>
-          <t>Lower-cost T2D combo</t>
+          <t>First oral GLP-1 for weight management</t>
         </is>
       </c>
       <c r="H76" s="26" t="inlineStr">
         <is>
-          <t>Lupin FDA approval April 8, 2026. Lower-cost combination for T2D management.</t>
+          <t>FDA approved late 2025/early 2026. First GLP-1 pill for weight loss. Launched in US Jan 2026.</t>
         </is>
       </c>
       <c r="I76" s="26" t="inlineStr">
         <is>
-          <t>FDA Approved (Generic)</t>
+          <t>FDA Approved</t>
         </is>
       </c>
       <c r="J76" s="26" t="n">
@@ -4756,335 +4756,225 @@
       </c>
       <c r="K76" s="26" t="inlineStr">
         <is>
-          <t>https://www.prismnews.com/news/lupin-wins-fda-approval-for-generic-dapagliflozin-metformin</t>
+          <t>https://www.ajmc.com/view/fda-approves-oral-semaglutide-as-first-glp-1-pill-for-weight-loss</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="26" t="inlineStr">
-        <is>
-          <t>Cross</t>
-        </is>
-      </c>
-      <c r="B77" s="26" t="inlineStr">
-        <is>
-          <t>GLP-1 - Oral</t>
-        </is>
-      </c>
-      <c r="C77" s="26" t="inlineStr">
-        <is>
-          <t>Oral Semaglutide 25mg (Wegovy)</t>
-        </is>
-      </c>
-      <c r="D77" s="26" t="inlineStr">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>Insulin</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>Awiqli (Insulin Icodec)</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
         <is>
           <t>Novo Nordisk</t>
         </is>
       </c>
-      <c r="E77" s="26" t="inlineStr">
-        <is>
-          <t>Oral GLP-1 RA for weight loss</t>
-        </is>
-      </c>
-      <c r="F77" s="26" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="G77" s="26" t="inlineStr">
-        <is>
-          <t>First oral GLP-1 for weight management</t>
-        </is>
-      </c>
-      <c r="H77" s="26" t="inlineStr">
-        <is>
-          <t>FDA approved late 2025/early 2026. First GLP-1 pill for weight loss. Launched in US Jan 2026.</t>
-        </is>
-      </c>
-      <c r="I77" s="26" t="inlineStr">
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>Once-weekly basal insulin</t>
+        </is>
+      </c>
+      <c r="F77" s="12" t="inlineStr">
         <is>
           <t>FDA Approved</t>
         </is>
       </c>
-      <c r="J77" s="26" t="n">
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>Glycemic control (weekly dosing)</t>
+        </is>
+      </c>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>FDA approved March 26, 2026. First weekly insulin. Reduces injections 365→52/yr. Based on 4 ONWARDS trials (n=2,680). T2D only.</t>
+        </is>
+      </c>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>FDA APPROVED</t>
+        </is>
+      </c>
+      <c r="J77" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K77" s="26" t="inlineStr">
-        <is>
-          <t>https://www.ajmc.com/view/fda-approves-oral-semaglutide-as-first-glp-1-pill-for-weight-loss</t>
+      <c r="K77" s="12" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/fda-approves-novo-nordisks-awiqli-the-first-and-only-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes-302726839.html</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>GLP-1 Agonist</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Orforglipron (Foundayo)</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Eli Lilly</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Oral non-peptide GLP-1 RA</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>SGLT2 Inhibitor</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="inlineStr">
+        <is>
+          <t>Generic Dapagliflozin (Farxiga)</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
+        <is>
+          <t>Multiple (Biocon, Lupin, others)</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>SGLT2 inhibitor (generic)</t>
+        </is>
+      </c>
+      <c r="F78" s="12" t="inlineStr">
         <is>
           <t>FDA Approved</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Weight loss / glycemic control</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>FDA approved April 1, 2026 for obesity/overweight. First oral small-molecule GLP-1 RA. No food/water restrictions.</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
+      <c r="G78" s="12" t="inlineStr">
+        <is>
+          <t>HF hospitalization / glycemic control</t>
+        </is>
+      </c>
+      <c r="H78" s="12" t="inlineStr">
+        <is>
+          <t>First SGLT2i generic approved April 7, 2026. 5mg and 10mg tablets. Major health equity milestone.</t>
+        </is>
+      </c>
+      <c r="I78" s="12" t="inlineStr">
         <is>
           <t>FDA APPROVED</t>
         </is>
       </c>
-      <c r="J78" t="n">
+      <c r="J78" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>https://investor.lilly.com/news-releases/news-release-details/fda-approves-lillys-foundayotm-orforglipron-only-glp-1-pill</t>
+      <c r="K78" s="12" t="inlineStr">
+        <is>
+          <t>https://www.fda.gov/drugs/drug-alerts-and-statements/fda-approves-first-generic-dapagliflozin-tablets</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>T2D</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Insulin</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Awiqli (Insulin Icodec)</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Novo Nordisk</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Once-weekly basal insulin</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>FDA Approved</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Glycemic control (weekly dosing)</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>FDA approved March 26, 2026. First weekly insulin. Reduces injections 365→52/yr. Based on 4 ONWARDS trials (n=2,680). T2D only.</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>FDA APPROVED</t>
-        </is>
-      </c>
-      <c r="J79" t="n">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>T1D/T2D</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>GLP-1 Pharmacogenomics</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>PAM Variant GLP-1 Resistance</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
+        <is>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>PAM enzyme variants reduce GLP-1 bioactivity</t>
+        </is>
+      </c>
+      <c r="F79" s="12" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="G79" s="12" t="inlineStr">
+        <is>
+          <t>Pharmacogenomics / precision medicine</t>
+        </is>
+      </c>
+      <c r="H79" s="12" t="inlineStr">
+        <is>
+          <t>~10% carry PAM variants causing GLP-1 resistance. Meta-analysis (n=1,119) showed lower HbA1c response. Genome Medicine, March 2026.</t>
+        </is>
+      </c>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>Published — Monitoring</t>
+        </is>
+      </c>
+      <c r="J79" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/fda-approves-novo-nordisks-awiqli-the-first-and-only-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes-302726839.html</t>
+      <c r="K79" s="12" t="inlineStr">
+        <is>
+          <t>https://med.stanford.edu/news/all-news/2026/04/glp-1-diabetes.html</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>T2D</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>SGLT2 Inhibitor</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Generic Dapagliflozin (Farxiga)</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Multiple (Biocon, Lupin, others)</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>SGLT2 inhibitor (generic)</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>FDA Approved</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>HF hospitalization / glycemic control</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>First SGLT2i generic approved April 7, 2026. 5mg and 10mg tablets. Major health equity milestone.</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>FDA APPROVED</t>
-        </is>
-      </c>
-      <c r="J80" t="n">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>T1D</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>GLP-1 — CV/Kidney</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>GLP-1 RA CV/Kidney Outcomes in T1D</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Bloomberg SPH</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>GLP-1 RA cardiorenal protection in T1D</t>
+        </is>
+      </c>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="inlineStr">
+        <is>
+          <t>CV event reduction / kidney protection</t>
+        </is>
+      </c>
+      <c r="H80" s="12" t="inlineStr">
+        <is>
+          <t>175K-patient study: 15% CV event reduction, 19% ESKD reduction, 16% mortality reduction in T1D. Nature Medicine, April 2026.</t>
+        </is>
+      </c>
+      <c r="I80" s="12" t="inlineStr">
+        <is>
+          <t>Published — Monitoring</t>
+        </is>
+      </c>
+      <c r="J80" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>https://www.fda.gov/drugs/drug-alerts-and-statements/fda-approves-first-generic-dapagliflozin-tablets</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>T1D/T2D</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>GLP-1 Pharmacogenomics</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>PAM Variant GLP-1 Resistance</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Stanford University</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>PAM enzyme variants reduce GLP-1 bioactivity</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Pharmacogenomics / precision medicine</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>~10% carry PAM variants causing GLP-1 resistance. Meta-analysis (n=1,119) showed lower HbA1c response. Genome Medicine, March 2026.</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>Published — Monitoring</t>
-        </is>
-      </c>
-      <c r="J81" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>https://med.stanford.edu/news/all-news/2026/04/glp-1-diabetes.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>T1D</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>GLP-1 — CV/Kidney</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>GLP-1 RA CV/Kidney Outcomes in T1D</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Johns Hopkins Bloomberg SPH</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>GLP-1 RA cardiorenal protection in T1D</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>CV event reduction / kidney protection</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>175K-patient study: 15% CV event reduction, 19% ESKD reduction, 16% mortality reduction in T1D. Nature Medicine, April 2026.</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Published — Monitoring</t>
-        </is>
-      </c>
-      <c r="J82" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K82" t="inlineStr">
+      <c r="K80" s="12" t="inlineStr">
         <is>
           <t>https://www.nature.com/articles/s41591-026-04274-0</t>
         </is>
@@ -8248,212 +8138,212 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Multi-tissue multi-omics integration reveals tissue-specific pathways, gene networks and drug candidates for type 1 diabetes</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>Blencowe M, Saleem Z, Liu R et al. (UCLA/Breakthrough T1D)</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>Diabetologia</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D45" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="12" t="inlineStr">
         <is>
           <t>Multi-Omics / Drug Repurposing</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="12" t="inlineStr">
         <is>
           <t>GWAS→network→drug screen identifies FYN, TAP1, LCK as key drivers; drug candidates validated against EMRs</t>
         </is>
       </c>
-      <c r="H45" t="n">
+      <c r="H45" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="12" t="inlineStr">
         <is>
           <t>Tier 1 alignment: Multi-Omics + Drug Repurposing. Cross-referenced with our islet repurposing analysis.</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s00125-026-06721-6</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>GLP-1 receptor agonists for major cardiovascular and kidney outcomes in type 1 diabetes</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>Johns Hopkins Bloomberg SPH</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>Nature Medicine</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D46" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="12" t="inlineStr">
         <is>
           <t>GLP-1 / Cardiovascular</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="12" t="inlineStr">
         <is>
           <t>175K-patient study: GLP-1 RAs reduce CV events 15%, ESKD 19% in T1D</t>
         </is>
       </c>
-      <c r="H46" t="n">
+      <c r="H46" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="12" t="inlineStr">
         <is>
           <t>Largest GLP-1 study in T1D. Links to NCT05819138.</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41591-026-04274-0</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>GLP-1 resistance: PAM enzyme variants reduce drug response in ~10% of people</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>Stanford University</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>Genome Medicine</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D47" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>T1D/T2D</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="12" t="inlineStr">
         <is>
           <t>Pharmacogenomics</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="12" t="inlineStr">
         <is>
           <t>PAM variants in ~10% of population cause reduced GLP-1 bioactivity and lower HbA1c response</t>
         </is>
       </c>
-      <c r="H47" t="n">
+      <c r="H47" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47" s="12" t="inlineStr">
         <is>
           <t>Novel GWAS/Polygenic × GLP-1 intersection. Suggests pharmacogenomics alert domain.</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="12" t="inlineStr">
         <is>
           <t>https://med.stanford.edu/news/all-news/2026/04/glp-1-diabetes.html</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="12" t="inlineStr">
         <is>
           <t>Dozens of AI disease-prediction models were trained on dubious data</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Basu M (reporting); Barnett A et al. (research)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D48" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="12" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="12" t="inlineStr">
         <is>
           <t>AI/ML Methodology</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="12" t="inlineStr">
         <is>
           <t>124 papers used potentially fabricated health datasets for ML training; some models may be in clinical use</t>
         </is>
       </c>
-      <c r="H48" t="n">
+      <c r="H48" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J48" s="12" t="inlineStr">
         <is>
           <t>Methodological caution for our AI/ML work. Added to Research Findings Summary.</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K48" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/d41586-026-00697-4</t>
         </is>

</xml_diff>